<commit_message>
chore: update WARN cache and subscriber data
</commit_message>
<xml_diff>
--- a/data/warn_report.xlsx
+++ b/data/warn_report.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\entshare3\JS-Data\WSB-CO\BPAC\Policy &amp; Program Communications Group\Communications Unit\Website Management\5. WARN (Worker Adjustment and Retraining Notification) Updates\2026\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C44EBC3E-62D9-4DB9-983F-1C5E29F52F64}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{693E3200-4D33-462B-A562-8625EDCF6BFD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="751" xr2:uid="{3EA4B9A5-CE9D-4ACF-B45F-4158810915D4}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5486" uniqueCount="1859">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5731" uniqueCount="1946">
   <si>
     <t>County/Parish</t>
   </si>
@@ -5645,6 +5645,135 @@
     <t>475 Anton Blvd.  Costa Mesa CA 92626</t>
   </si>
   <si>
+    <t>Sanitation Specialists</t>
+  </si>
+  <si>
+    <t>14490 Catalina Street  San Leandro CA 94577</t>
+  </si>
+  <si>
+    <t>Union of Pan Asian Communities (Neighborhood Enterprise Center)</t>
+  </si>
+  <si>
+    <t>5296 University Avenue  San Diego CA 92105</t>
+  </si>
+  <si>
+    <t>Atlassian US, Inc.</t>
+  </si>
+  <si>
+    <t>350 Bush Street, Floor 13  San Francisco CA 94104</t>
+  </si>
+  <si>
+    <t>320B Shaw Road  South San Francisco CA 94080</t>
+  </si>
+  <si>
+    <t>American Eagle Flights (Santa Maria Airport)</t>
+  </si>
+  <si>
+    <t>3217 Terminal Dr.  Santa Maria CA 93455</t>
+  </si>
+  <si>
+    <t>Westside Equipment Co. (OXBO)</t>
+  </si>
+  <si>
+    <t>18 Fink Road  Crows Landing CA 95313</t>
+  </si>
+  <si>
+    <t>Blue Shield of California</t>
+  </si>
+  <si>
+    <t>Blue Shield of California (Building C)</t>
+  </si>
+  <si>
+    <t>4203 Town Center Blvd., Building C  El Dorado Hills CA 95762</t>
+  </si>
+  <si>
+    <t>Blue Shield of California (Building B)</t>
+  </si>
+  <si>
+    <t>4203 Town Center Blvd., Building B  El Dorado Hills CA 95762</t>
+  </si>
+  <si>
+    <t>Calvary Murrieta Christian School</t>
+  </si>
+  <si>
+    <t>2475 Monroe Avenue  Murrieta CA 92562</t>
+  </si>
+  <si>
+    <t>Heritage Bank of Commerce (Livermore)</t>
+  </si>
+  <si>
+    <t>1987 First Street  Livermore CA 94550</t>
+  </si>
+  <si>
+    <t>Heritage Bank of Commerce (Oakland)</t>
+  </si>
+  <si>
+    <t>1111 Broadway, Suite 1650  Oakland CA 94607</t>
+  </si>
+  <si>
+    <t>Heritage Bank of Commerce (Danville)</t>
+  </si>
+  <si>
+    <t>387 Diable Blvd.  Danville CA 94526</t>
+  </si>
+  <si>
+    <t>Heritage Bank of Commerce (Walnut Creek)</t>
+  </si>
+  <si>
+    <t>1990 N. California Blvd, Suite 100  Walnut Creek CA 94596</t>
+  </si>
+  <si>
+    <t>Heritage Bank of Commerce (San Rafael)</t>
+  </si>
+  <si>
+    <t>999 Fifth Ave., Suite 100  San Rafael CA 94901</t>
+  </si>
+  <si>
+    <t>San Benito County</t>
+  </si>
+  <si>
+    <t>Heritage Bank of Commerce (Hollister)</t>
+  </si>
+  <si>
+    <t>351 Tres Pinos Road, Suite 102A  Hollister CA 95023</t>
+  </si>
+  <si>
+    <t>Heritage Bank of Commerce (San Francisco)</t>
+  </si>
+  <si>
+    <t>120 Kearney St., Suite 2300  San Francisco CA 94108</t>
+  </si>
+  <si>
+    <t>Heritage Bank of Commerce (Mateo)</t>
+  </si>
+  <si>
+    <t>400 S. El Camino Real, Suite 150  Mateo CA 94402</t>
+  </si>
+  <si>
+    <t>Heritage Bank of Commerce (Los Altos)</t>
+  </si>
+  <si>
+    <t>419 South San Antonio Road  Los Altos CA 94022</t>
+  </si>
+  <si>
+    <t>Heritage Bank of Commerce (Morgan Hill)</t>
+  </si>
+  <si>
+    <t>18625 Sutter Blvd. Suite 100  Morgan Hill CA 95037</t>
+  </si>
+  <si>
+    <t>Heritage Bank of Commerce (Remote-San Jose)</t>
+  </si>
+  <si>
+    <t>224 Airport Parkway  San Jose CA 95110</t>
+  </si>
+  <si>
+    <t>Heritage Bank of Commerce (San Jose)</t>
+  </si>
+  <si>
+    <t>Experian (Experian Health and Experian Information Solutions)</t>
+  </si>
+  <si>
     <r>
       <rPr>
         <b/>
@@ -5664,7 +5793,7 @@
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve">
-01/01/2023 - 03/16/2026
+01/01/2023 - 03/23/2026
 </t>
     </r>
     <r>
@@ -5678,58 +5807,190 @@
     </r>
   </si>
   <si>
-    <t>Sanitation Specialists</t>
-  </si>
-  <si>
-    <t>14490 Catalina Street  San Leandro CA 94577</t>
-  </si>
-  <si>
-    <t>Union of Pan Asian Communities (Neighborhood Enterprise Center)</t>
-  </si>
-  <si>
-    <t>5296 University Avenue  San Diego CA 92105</t>
-  </si>
-  <si>
-    <t>Atlassian US, Inc.</t>
-  </si>
-  <si>
-    <t>350 Bush Street, Floor 13  San Francisco CA 94104</t>
-  </si>
-  <si>
-    <t>320B Shaw Road  South San Francisco CA 94080</t>
-  </si>
-  <si>
-    <t>American Eagle Flights (Santa Maria Airport)</t>
-  </si>
-  <si>
-    <t>3217 Terminal Dr.  Santa Maria CA 93455</t>
-  </si>
-  <si>
-    <t>Westside Equipment Co. (OXBO)</t>
-  </si>
-  <si>
-    <t>18 Fink Road  Crows Landing CA 95313</t>
-  </si>
-  <si>
-    <t>Blue Shield of California</t>
-  </si>
-  <si>
-    <t>Blue Shield of California (Building C)</t>
-  </si>
-  <si>
-    <t>4203 Town Center Blvd., Building C  El Dorado Hills CA 95762</t>
-  </si>
-  <si>
-    <t>Blue Shield of California (Building B)</t>
-  </si>
-  <si>
-    <t>4203 Town Center Blvd., Building B  El Dorado Hills CA 95762</t>
-  </si>
-  <si>
-    <t>Calvary Murrieta Christian School</t>
-  </si>
-  <si>
-    <t>2475 Monroe Avenue  Murrieta CA 92562</t>
+    <t>Total Storage Solutions (Best RV &amp; Self Storage)</t>
+  </si>
+  <si>
+    <t>5900 Esperanza Ave.  Whittier CA 90606</t>
+  </si>
+  <si>
+    <t>Total Storage Solutions (Crenshaw Self Storage)</t>
+  </si>
+  <si>
+    <t>6725 Crenshaw Blvd.  Los Angeles CA 90043</t>
+  </si>
+  <si>
+    <t>Total Storage Solutions (El Monte Stor It Now)</t>
+  </si>
+  <si>
+    <t>10212 Valley Blvd.  El Monte CA 91731</t>
+  </si>
+  <si>
+    <t>Total Storage Solutions (Studebaker Self Storage)</t>
+  </si>
+  <si>
+    <t>698 N. Studebaker Rd.  Long Beach CA 90803</t>
+  </si>
+  <si>
+    <t>Total Storage Solutions (Arcadia 210 Self Storage)</t>
+  </si>
+  <si>
+    <t>324 N. 2nd Ave.  Arcadia CA 91006</t>
+  </si>
+  <si>
+    <t>Total Storage Solutions (All Size Self Storage)</t>
+  </si>
+  <si>
+    <t>911 Calle Amanecer  San Clemente CA 92673</t>
+  </si>
+  <si>
+    <t>Total Storage Solutions (All Size Laguna Niguel)</t>
+  </si>
+  <si>
+    <t>27872 Crown Valley Parkway  Laguna Niguel CA 92677</t>
+  </si>
+  <si>
+    <t>Total Storage Solutions (Garden Grove Secured Storage)</t>
+  </si>
+  <si>
+    <t>13632 S. Euclid St.  Garden Grove CA 92843</t>
+  </si>
+  <si>
+    <t>Total Storage Solutions (Townsend Self Storage)</t>
+  </si>
+  <si>
+    <t>308 N. Townsend St.  Santa Ana CA 92703</t>
+  </si>
+  <si>
+    <t>Total Storage Solutions (Airport Mini Storage)</t>
+  </si>
+  <si>
+    <t>7044 Arlington Ave.  Riverside CA 92503</t>
+  </si>
+  <si>
+    <t>Total Storage Solutions (Aware Self Storage)</t>
+  </si>
+  <si>
+    <t>5021 W. Ramsey St.  Banning CA 92220</t>
+  </si>
+  <si>
+    <t>Total Storage Solutions (Beaumont RV &amp; Self Storage)</t>
+  </si>
+  <si>
+    <t>251 W. 1st St.  Beaumont CA 92223</t>
+  </si>
+  <si>
+    <t>Total Storage Solutions (Beaumont Self Storage)</t>
+  </si>
+  <si>
+    <t>190 E. First St.  Beaumont CA 92223</t>
+  </si>
+  <si>
+    <t>Total Storage Solutions (Jefferson Self Storage)</t>
+  </si>
+  <si>
+    <t>25435 Jefferson Ave.  Murrieta CA 92562</t>
+  </si>
+  <si>
+    <t>Total Storage Solutions (Sun City Mini Storage)</t>
+  </si>
+  <si>
+    <t>27460 McCall Blvd.  Sun City CA 92585</t>
+  </si>
+  <si>
+    <t>Total Storage Solutions (Tri-City Self Storage)</t>
+  </si>
+  <si>
+    <t>485 W. LaCadena  Riverside CA 92501</t>
+  </si>
+  <si>
+    <t>Total Storage Solutions (Western States Self Storage)</t>
+  </si>
+  <si>
+    <t>23190 Hemlock Ave.  Moreno Valley CA 92557</t>
+  </si>
+  <si>
+    <t>Total Storage Solutions (Riverside Self Storage)</t>
+  </si>
+  <si>
+    <t>7200 Indiana Ave.  Riverside CA 92504</t>
+  </si>
+  <si>
+    <t>Total Storage Solutions (E Street Self Storage)</t>
+  </si>
+  <si>
+    <t>1723 S. E St.  San Bernardino CA 92408</t>
+  </si>
+  <si>
+    <t>Total Storage Solutions (Citrus Plaza Self Storage)</t>
+  </si>
+  <si>
+    <t>202 W. College St., Suite 100  Fallbrook CA 92028</t>
+  </si>
+  <si>
+    <t>Lodging Dynamics Hospitality Group, LLC (Courtyard &amp; TownePlace Suites)</t>
+  </si>
+  <si>
+    <t>4427 West El Segundo  Hawthorne CA 90250</t>
+  </si>
+  <si>
+    <t>Lodging Dynamics Hospitality Group, LLC (Midici Restaurant)</t>
+  </si>
+  <si>
+    <t>Lodging Dynamics Hospitality Group, LLC (Hilton Garden Inn)</t>
+  </si>
+  <si>
+    <t>2410 Marine Avenue  Redondo Beach CA 90278</t>
+  </si>
+  <si>
+    <t>Lodging Dynamics Hospitality Group, LLC (Residence Inn)</t>
+  </si>
+  <si>
+    <t>2420 Marine Avenue  Redondo Beach CA 90278</t>
+  </si>
+  <si>
+    <t>Lodging Dynamics Hospitality Group, LLC (Homewood Suites)</t>
+  </si>
+  <si>
+    <t>2430 Marine Avenue  Redondo Beach CA 90278</t>
+  </si>
+  <si>
+    <t>NSI-Lynn Electronics</t>
+  </si>
+  <si>
+    <t>3162 East La Palma Avenue  Anaheim CA 92806</t>
+  </si>
+  <si>
+    <t>ERN Services, Inc.</t>
+  </si>
+  <si>
+    <t>5757 Century Bl. Suite 752  Los Angeles CA 90045</t>
+  </si>
+  <si>
+    <t>Waymakers</t>
+  </si>
+  <si>
+    <t>440 Exchange, Ste. 250 and 200  Irvine CA 92602</t>
+  </si>
+  <si>
+    <t>16580 Harbor Blvd., Unit O  Fountain Valley CA 92708</t>
+  </si>
+  <si>
+    <t>City National Bank (555 S. Flower Street)</t>
+  </si>
+  <si>
+    <t>555 S. Flower Street  Los Angeles CA 90071</t>
+  </si>
+  <si>
+    <t>City National Bank (350 S. Grand Ave.)</t>
+  </si>
+  <si>
+    <t>675 Almanor Ave  Sunnyvale CA 94085</t>
+  </si>
+  <si>
+    <t>Summit Funding, Inc.</t>
+  </si>
+  <si>
+    <t>2135 Butano Drive, #150  Sacramento CA 95825</t>
   </si>
   <si>
     <r>
@@ -5743,7 +6004,7 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t>07/01/25 to 03/16/2026</t>
+      <t>07/01/25 to 03/23/2026</t>
     </r>
     <r>
       <rPr>
@@ -5763,7 +6024,7 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t>A detailed WARN summary by county and filtered according to processed date. Table Spans cells A2 through I1085.</t>
+      <t>A detailed WARN summary by county and filtered according to processed date. Table Spans cells A2 through I1134.</t>
     </r>
   </si>
 </sst>
@@ -6113,7 +6374,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="55">
+  <cellXfs count="56">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -6270,6 +6531,9 @@
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="14" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1" readingOrder="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="4">
@@ -7062,7 +7326,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{1F69E8FD-21FF-4B81-951D-D7EC70F8E5F9}" name="DetailedWarnReport" displayName="DetailedWarnReport" ref="A2:I1085" totalsRowShown="0" headerRowDxfId="31" dataDxfId="30">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{1F69E8FD-21FF-4B81-951D-D7EC70F8E5F9}" name="DetailedWarnReport" displayName="DetailedWarnReport" ref="A2:I1134" totalsRowShown="0" headerRowDxfId="31" dataDxfId="30">
   <tableColumns count="9">
     <tableColumn id="1" xr3:uid="{3E60720E-46D7-48F7-AF17-837D42D08A11}" name="County/Parish" dataDxfId="29"/>
     <tableColumn id="2" xr3:uid="{058DED91-D77E-48B6-A71D-06D4A25AA391}" name="Notice_x000a_Date" dataDxfId="28"/>
@@ -7458,7 +7722,7 @@
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="28.42578125" style="3" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="6.42578125" style="3" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="6.5703125" style="3" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="78.75" x14ac:dyDescent="0.25">
@@ -7480,7 +7744,7 @@
       </c>
       <c r="B3" s="11">
         <f>SUM('Detailed WARN Report '!G:G)</f>
-        <v>59245</v>
+        <v>60159</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
@@ -7514,7 +7778,7 @@
       </c>
       <c r="B7" s="11">
         <f>COUNTIF('Detailed WARN Report '!F:F,"Closure Permanent")</f>
-        <v>297</v>
+        <v>299</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
@@ -7545,7 +7809,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D3E7117B-AC46-45AC-B2F3-AE611FA82488}">
-  <dimension ref="A1:I1085"/>
+  <dimension ref="A1:I1134"/>
   <sheetFormatPr defaultColWidth="161.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="29" style="3" bestFit="1" customWidth="1"/>
@@ -7561,7 +7825,7 @@
   <sheetData>
     <row r="1" spans="1:9" ht="102" x14ac:dyDescent="0.25">
       <c r="A1" s="16" t="s">
-        <v>1858</v>
+        <v>1945</v>
       </c>
       <c r="E1" s="3"/>
     </row>
@@ -38551,7 +38815,7 @@
         <v>46164</v>
       </c>
       <c r="E1070" s="37" t="s">
-        <v>1840</v>
+        <v>1839</v>
       </c>
       <c r="F1070" s="37" t="s">
         <v>54</v>
@@ -38560,7 +38824,7 @@
         <v>21</v>
       </c>
       <c r="H1070" s="34" t="s">
-        <v>1841</v>
+        <v>1840</v>
       </c>
       <c r="I1070" s="26" t="s">
         <v>43</v>
@@ -38580,7 +38844,7 @@
         <v>46152</v>
       </c>
       <c r="E1071" s="37" t="s">
-        <v>1842</v>
+        <v>1841</v>
       </c>
       <c r="F1071" s="37" t="s">
         <v>54</v>
@@ -38589,7 +38853,7 @@
         <v>16</v>
       </c>
       <c r="H1071" s="34" t="s">
-        <v>1843</v>
+        <v>1842</v>
       </c>
       <c r="I1071" s="26" t="s">
         <v>45</v>
@@ -38609,7 +38873,7 @@
         <v>46094</v>
       </c>
       <c r="E1072" s="37" t="s">
-        <v>1844</v>
+        <v>1843</v>
       </c>
       <c r="F1072" s="37" t="s">
         <v>6</v>
@@ -38618,7 +38882,7 @@
         <v>252</v>
       </c>
       <c r="H1072" s="34" t="s">
-        <v>1845</v>
+        <v>1844</v>
       </c>
       <c r="I1072" s="26" t="s">
         <v>41</v>
@@ -38638,7 +38902,7 @@
         <v>46164</v>
       </c>
       <c r="E1073" s="37" t="s">
-        <v>1840</v>
+        <v>1839</v>
       </c>
       <c r="F1073" s="37" t="s">
         <v>54</v>
@@ -38647,7 +38911,7 @@
         <v>15</v>
       </c>
       <c r="H1073" s="34" t="s">
-        <v>1846</v>
+        <v>1845</v>
       </c>
       <c r="I1073" s="26" t="s">
         <v>43</v>
@@ -38667,7 +38931,7 @@
         <v>46148</v>
       </c>
       <c r="E1074" s="37" t="s">
-        <v>1847</v>
+        <v>1846</v>
       </c>
       <c r="F1074" s="37" t="s">
         <v>54</v>
@@ -38676,7 +38940,7 @@
         <v>20</v>
       </c>
       <c r="H1074" s="34" t="s">
-        <v>1848</v>
+        <v>1847</v>
       </c>
       <c r="I1074" s="26" t="s">
         <v>37</v>
@@ -38696,7 +38960,7 @@
         <v>46153</v>
       </c>
       <c r="E1075" s="37" t="s">
-        <v>1849</v>
+        <v>1848</v>
       </c>
       <c r="F1075" s="37" t="s">
         <v>54</v>
@@ -38705,7 +38969,7 @@
         <v>2</v>
       </c>
       <c r="H1075" s="34" t="s">
-        <v>1850</v>
+        <v>1849</v>
       </c>
       <c r="I1075" s="26" t="s">
         <v>34</v>
@@ -38725,7 +38989,7 @@
         <v>46120</v>
       </c>
       <c r="E1076" s="37" t="s">
-        <v>1851</v>
+        <v>1850</v>
       </c>
       <c r="F1076" s="37" t="s">
         <v>6</v>
@@ -38754,7 +39018,7 @@
         <v>46120</v>
       </c>
       <c r="E1077" s="37" t="s">
-        <v>1852</v>
+        <v>1851</v>
       </c>
       <c r="F1077" s="37" t="s">
         <v>6</v>
@@ -38763,7 +39027,7 @@
         <v>5</v>
       </c>
       <c r="H1077" s="34" t="s">
-        <v>1853</v>
+        <v>1852</v>
       </c>
       <c r="I1077" s="26" t="s">
         <v>39</v>
@@ -38783,7 +39047,7 @@
         <v>46120</v>
       </c>
       <c r="E1078" s="37" t="s">
-        <v>1854</v>
+        <v>1853</v>
       </c>
       <c r="F1078" s="37" t="s">
         <v>6</v>
@@ -38792,7 +39056,7 @@
         <v>7</v>
       </c>
       <c r="H1078" s="34" t="s">
-        <v>1855</v>
+        <v>1854</v>
       </c>
       <c r="I1078" s="26" t="s">
         <v>39</v>
@@ -38812,7 +39076,7 @@
         <v>46120</v>
       </c>
       <c r="E1079" s="37" t="s">
-        <v>1851</v>
+        <v>1850</v>
       </c>
       <c r="F1079" s="37" t="s">
         <v>6</v>
@@ -38841,7 +39105,7 @@
         <v>46120</v>
       </c>
       <c r="E1080" s="37" t="s">
-        <v>1851</v>
+        <v>1850</v>
       </c>
       <c r="F1080" s="37" t="s">
         <v>6</v>
@@ -38870,7 +39134,7 @@
         <v>46120</v>
       </c>
       <c r="E1081" s="37" t="s">
-        <v>1851</v>
+        <v>1850</v>
       </c>
       <c r="F1081" s="37" t="s">
         <v>6</v>
@@ -38899,7 +39163,7 @@
         <v>46120</v>
       </c>
       <c r="E1082" s="37" t="s">
-        <v>1851</v>
+        <v>1850</v>
       </c>
       <c r="F1082" s="37" t="s">
         <v>6</v>
@@ -38928,7 +39192,7 @@
         <v>46120</v>
       </c>
       <c r="E1083" s="37" t="s">
-        <v>1851</v>
+        <v>1850</v>
       </c>
       <c r="F1083" s="37" t="s">
         <v>6</v>
@@ -38957,7 +39221,7 @@
         <v>46120</v>
       </c>
       <c r="E1084" s="37" t="s">
-        <v>1851</v>
+        <v>1850</v>
       </c>
       <c r="F1084" s="37" t="s">
         <v>6</v>
@@ -38986,7 +39250,7 @@
         <v>46171</v>
       </c>
       <c r="E1085" s="41" t="s">
-        <v>1856</v>
+        <v>1855</v>
       </c>
       <c r="F1085" s="41" t="s">
         <v>54</v>
@@ -38995,10 +39259,1431 @@
         <v>74</v>
       </c>
       <c r="H1085" s="34" t="s">
-        <v>1857</v>
+        <v>1856</v>
       </c>
       <c r="I1085" s="26" t="s">
         <v>44</v>
+      </c>
+    </row>
+    <row r="1086" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1086" s="35" t="s">
+        <v>198</v>
+      </c>
+      <c r="B1086" s="36">
+        <v>46098</v>
+      </c>
+      <c r="C1086" s="36">
+        <v>46098</v>
+      </c>
+      <c r="D1086" s="48">
+        <v>46178</v>
+      </c>
+      <c r="E1086" s="32" t="s">
+        <v>199</v>
+      </c>
+      <c r="F1086" s="32" t="s">
+        <v>6</v>
+      </c>
+      <c r="G1086" s="34">
+        <v>3</v>
+      </c>
+      <c r="H1086" s="34" t="s">
+        <v>200</v>
+      </c>
+      <c r="I1086" s="26" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="1087" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1087" s="35" t="s">
+        <v>52</v>
+      </c>
+      <c r="B1087" s="36">
+        <v>46080</v>
+      </c>
+      <c r="C1087" s="36">
+        <v>46098</v>
+      </c>
+      <c r="D1087" s="48">
+        <v>46129</v>
+      </c>
+      <c r="E1087" s="32" t="s">
+        <v>1857</v>
+      </c>
+      <c r="F1087" s="32" t="s">
+        <v>6</v>
+      </c>
+      <c r="G1087" s="34">
+        <v>1</v>
+      </c>
+      <c r="H1087" s="34" t="s">
+        <v>1858</v>
+      </c>
+      <c r="I1087" s="26" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="1088" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1088" s="35" t="s">
+        <v>52</v>
+      </c>
+      <c r="B1088" s="36">
+        <v>46080</v>
+      </c>
+      <c r="C1088" s="36">
+        <v>46098</v>
+      </c>
+      <c r="D1088" s="48">
+        <v>46129</v>
+      </c>
+      <c r="E1088" s="32" t="s">
+        <v>1859</v>
+      </c>
+      <c r="F1088" s="32" t="s">
+        <v>6</v>
+      </c>
+      <c r="G1088" s="34">
+        <v>1</v>
+      </c>
+      <c r="H1088" s="34" t="s">
+        <v>1860</v>
+      </c>
+      <c r="I1088" s="26" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="1089" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1089" s="35" t="s">
+        <v>198</v>
+      </c>
+      <c r="B1089" s="36">
+        <v>46080</v>
+      </c>
+      <c r="C1089" s="36">
+        <v>46098</v>
+      </c>
+      <c r="D1089" s="48">
+        <v>46129</v>
+      </c>
+      <c r="E1089" s="32" t="s">
+        <v>1861</v>
+      </c>
+      <c r="F1089" s="32" t="s">
+        <v>6</v>
+      </c>
+      <c r="G1089" s="34">
+        <v>4</v>
+      </c>
+      <c r="H1089" s="34" t="s">
+        <v>1862</v>
+      </c>
+      <c r="I1089" s="26" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="1090" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1090" s="35" t="s">
+        <v>198</v>
+      </c>
+      <c r="B1090" s="36">
+        <v>46080</v>
+      </c>
+      <c r="C1090" s="36">
+        <v>46098</v>
+      </c>
+      <c r="D1090" s="48">
+        <v>46129</v>
+      </c>
+      <c r="E1090" s="32" t="s">
+        <v>1863</v>
+      </c>
+      <c r="F1090" s="32" t="s">
+        <v>6</v>
+      </c>
+      <c r="G1090" s="34">
+        <v>4</v>
+      </c>
+      <c r="H1090" s="34" t="s">
+        <v>1864</v>
+      </c>
+      <c r="I1090" s="26" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="1091" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1091" s="35" t="s">
+        <v>285</v>
+      </c>
+      <c r="B1091" s="36">
+        <v>46080</v>
+      </c>
+      <c r="C1091" s="36">
+        <v>46098</v>
+      </c>
+      <c r="D1091" s="48">
+        <v>46129</v>
+      </c>
+      <c r="E1091" s="32" t="s">
+        <v>1865</v>
+      </c>
+      <c r="F1091" s="32" t="s">
+        <v>6</v>
+      </c>
+      <c r="G1091" s="34">
+        <v>3</v>
+      </c>
+      <c r="H1091" s="34" t="s">
+        <v>1866</v>
+      </c>
+      <c r="I1091" s="26" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="1092" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1092" s="35" t="s">
+        <v>1867</v>
+      </c>
+      <c r="B1092" s="36">
+        <v>46080</v>
+      </c>
+      <c r="C1092" s="36">
+        <v>46098</v>
+      </c>
+      <c r="D1092" s="48">
+        <v>46129</v>
+      </c>
+      <c r="E1092" s="32" t="s">
+        <v>1868</v>
+      </c>
+      <c r="F1092" s="32" t="s">
+        <v>6</v>
+      </c>
+      <c r="G1092" s="34">
+        <v>1</v>
+      </c>
+      <c r="H1092" s="34" t="s">
+        <v>1869</v>
+      </c>
+      <c r="I1092" s="26" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="1093" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1093" s="35" t="s">
+        <v>94</v>
+      </c>
+      <c r="B1093" s="36">
+        <v>46080</v>
+      </c>
+      <c r="C1093" s="36">
+        <v>46098</v>
+      </c>
+      <c r="D1093" s="48">
+        <v>46129</v>
+      </c>
+      <c r="E1093" s="32" t="s">
+        <v>1870</v>
+      </c>
+      <c r="F1093" s="32" t="s">
+        <v>6</v>
+      </c>
+      <c r="G1093" s="34">
+        <v>3</v>
+      </c>
+      <c r="H1093" s="34" t="s">
+        <v>1871</v>
+      </c>
+      <c r="I1093" s="26" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="1094" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1094" s="35" t="s">
+        <v>97</v>
+      </c>
+      <c r="B1094" s="36">
+        <v>46080</v>
+      </c>
+      <c r="C1094" s="36">
+        <v>46098</v>
+      </c>
+      <c r="D1094" s="48">
+        <v>46129</v>
+      </c>
+      <c r="E1094" s="32" t="s">
+        <v>1872</v>
+      </c>
+      <c r="F1094" s="32" t="s">
+        <v>6</v>
+      </c>
+      <c r="G1094" s="34">
+        <v>5</v>
+      </c>
+      <c r="H1094" s="34" t="s">
+        <v>1873</v>
+      </c>
+      <c r="I1094" s="26" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="1095" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1095" s="35" t="s">
+        <v>90</v>
+      </c>
+      <c r="B1095" s="36">
+        <v>46080</v>
+      </c>
+      <c r="C1095" s="36">
+        <v>46098</v>
+      </c>
+      <c r="D1095" s="48">
+        <v>46129</v>
+      </c>
+      <c r="E1095" s="32" t="s">
+        <v>1874</v>
+      </c>
+      <c r="F1095" s="32" t="s">
+        <v>6</v>
+      </c>
+      <c r="G1095" s="34">
+        <v>1</v>
+      </c>
+      <c r="H1095" s="34" t="s">
+        <v>1875</v>
+      </c>
+      <c r="I1095" s="26" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="1096" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1096" s="35" t="s">
+        <v>90</v>
+      </c>
+      <c r="B1096" s="36">
+        <v>46080</v>
+      </c>
+      <c r="C1096" s="36">
+        <v>46098</v>
+      </c>
+      <c r="D1096" s="48">
+        <v>46129</v>
+      </c>
+      <c r="E1096" s="32" t="s">
+        <v>1876</v>
+      </c>
+      <c r="F1096" s="32" t="s">
+        <v>6</v>
+      </c>
+      <c r="G1096" s="34">
+        <v>1</v>
+      </c>
+      <c r="H1096" s="34" t="s">
+        <v>1877</v>
+      </c>
+      <c r="I1096" s="26" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="1097" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1097" s="35" t="s">
+        <v>90</v>
+      </c>
+      <c r="B1097" s="36">
+        <v>46080</v>
+      </c>
+      <c r="C1097" s="36">
+        <v>46098</v>
+      </c>
+      <c r="D1097" s="48">
+        <v>46129</v>
+      </c>
+      <c r="E1097" s="32" t="s">
+        <v>1878</v>
+      </c>
+      <c r="F1097" s="32" t="s">
+        <v>6</v>
+      </c>
+      <c r="G1097" s="34">
+        <v>12</v>
+      </c>
+      <c r="H1097" s="34" t="s">
+        <v>1879</v>
+      </c>
+      <c r="I1097" s="26" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="1098" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1098" s="35" t="s">
+        <v>90</v>
+      </c>
+      <c r="B1098" s="36">
+        <v>46080</v>
+      </c>
+      <c r="C1098" s="36">
+        <v>46098</v>
+      </c>
+      <c r="D1098" s="48">
+        <v>46129</v>
+      </c>
+      <c r="E1098" s="32" t="s">
+        <v>1880</v>
+      </c>
+      <c r="F1098" s="32" t="s">
+        <v>6</v>
+      </c>
+      <c r="G1098" s="34">
+        <v>85</v>
+      </c>
+      <c r="H1098" s="34" t="s">
+        <v>1879</v>
+      </c>
+      <c r="I1098" s="26" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="1099" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1099" s="39" t="s">
+        <v>64</v>
+      </c>
+      <c r="B1099" s="40">
+        <v>46098</v>
+      </c>
+      <c r="C1099" s="40">
+        <v>46098</v>
+      </c>
+      <c r="D1099" s="55">
+        <v>46160</v>
+      </c>
+      <c r="E1099" s="32" t="s">
+        <v>1881</v>
+      </c>
+      <c r="F1099" s="32" t="s">
+        <v>6</v>
+      </c>
+      <c r="G1099" s="34">
+        <v>5</v>
+      </c>
+      <c r="H1099" s="34" t="s">
+        <v>1838</v>
+      </c>
+      <c r="I1099" s="26" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="1100" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1100" s="35" t="s">
+        <v>5</v>
+      </c>
+      <c r="B1100" s="36">
+        <v>46093</v>
+      </c>
+      <c r="C1100" s="36">
+        <v>46100</v>
+      </c>
+      <c r="D1100" s="48">
+        <v>46160</v>
+      </c>
+      <c r="E1100" s="32" t="s">
+        <v>1883</v>
+      </c>
+      <c r="F1100" s="32" t="s">
+        <v>6</v>
+      </c>
+      <c r="G1100" s="34">
+        <v>3</v>
+      </c>
+      <c r="H1100" s="34" t="s">
+        <v>1884</v>
+      </c>
+      <c r="I1100" s="26" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="1101" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1101" s="35" t="s">
+        <v>5</v>
+      </c>
+      <c r="B1101" s="36">
+        <v>46093</v>
+      </c>
+      <c r="C1101" s="36">
+        <v>46100</v>
+      </c>
+      <c r="D1101" s="48">
+        <v>46160</v>
+      </c>
+      <c r="E1101" s="32" t="s">
+        <v>1885</v>
+      </c>
+      <c r="F1101" s="32" t="s">
+        <v>6</v>
+      </c>
+      <c r="G1101" s="34">
+        <v>2</v>
+      </c>
+      <c r="H1101" s="34" t="s">
+        <v>1886</v>
+      </c>
+      <c r="I1101" s="26" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="1102" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1102" s="35" t="s">
+        <v>5</v>
+      </c>
+      <c r="B1102" s="36">
+        <v>46093</v>
+      </c>
+      <c r="C1102" s="36">
+        <v>46100</v>
+      </c>
+      <c r="D1102" s="48">
+        <v>46160</v>
+      </c>
+      <c r="E1102" s="32" t="s">
+        <v>1887</v>
+      </c>
+      <c r="F1102" s="32" t="s">
+        <v>6</v>
+      </c>
+      <c r="G1102" s="34">
+        <v>3</v>
+      </c>
+      <c r="H1102" s="34" t="s">
+        <v>1888</v>
+      </c>
+      <c r="I1102" s="26" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="1103" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1103" s="35" t="s">
+        <v>5</v>
+      </c>
+      <c r="B1103" s="36">
+        <v>46093</v>
+      </c>
+      <c r="C1103" s="36">
+        <v>46100</v>
+      </c>
+      <c r="D1103" s="48">
+        <v>46160</v>
+      </c>
+      <c r="E1103" s="32" t="s">
+        <v>1889</v>
+      </c>
+      <c r="F1103" s="32" t="s">
+        <v>6</v>
+      </c>
+      <c r="G1103" s="34">
+        <v>3</v>
+      </c>
+      <c r="H1103" s="34" t="s">
+        <v>1890</v>
+      </c>
+      <c r="I1103" s="26" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="1104" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1104" s="35" t="s">
+        <v>5</v>
+      </c>
+      <c r="B1104" s="36">
+        <v>46093</v>
+      </c>
+      <c r="C1104" s="36">
+        <v>46100</v>
+      </c>
+      <c r="D1104" s="48">
+        <v>46160</v>
+      </c>
+      <c r="E1104" s="32" t="s">
+        <v>1891</v>
+      </c>
+      <c r="F1104" s="32" t="s">
+        <v>6</v>
+      </c>
+      <c r="G1104" s="34">
+        <v>1</v>
+      </c>
+      <c r="H1104" s="34" t="s">
+        <v>1892</v>
+      </c>
+      <c r="I1104" s="26" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="1105" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1105" s="35" t="s">
+        <v>64</v>
+      </c>
+      <c r="B1105" s="36">
+        <v>46093</v>
+      </c>
+      <c r="C1105" s="36">
+        <v>46100</v>
+      </c>
+      <c r="D1105" s="48">
+        <v>46160</v>
+      </c>
+      <c r="E1105" s="32" t="s">
+        <v>1893</v>
+      </c>
+      <c r="F1105" s="32" t="s">
+        <v>6</v>
+      </c>
+      <c r="G1105" s="34">
+        <v>3</v>
+      </c>
+      <c r="H1105" s="34" t="s">
+        <v>1894</v>
+      </c>
+      <c r="I1105" s="26" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="1106" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1106" s="35" t="s">
+        <v>64</v>
+      </c>
+      <c r="B1106" s="36">
+        <v>46093</v>
+      </c>
+      <c r="C1106" s="36">
+        <v>46100</v>
+      </c>
+      <c r="D1106" s="48">
+        <v>46160</v>
+      </c>
+      <c r="E1106" s="32" t="s">
+        <v>1895</v>
+      </c>
+      <c r="F1106" s="32" t="s">
+        <v>6</v>
+      </c>
+      <c r="G1106" s="34">
+        <v>3</v>
+      </c>
+      <c r="H1106" s="34" t="s">
+        <v>1896</v>
+      </c>
+      <c r="I1106" s="26" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="1107" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1107" s="35" t="s">
+        <v>64</v>
+      </c>
+      <c r="B1107" s="36">
+        <v>46093</v>
+      </c>
+      <c r="C1107" s="36">
+        <v>46100</v>
+      </c>
+      <c r="D1107" s="48">
+        <v>46160</v>
+      </c>
+      <c r="E1107" s="32" t="s">
+        <v>1897</v>
+      </c>
+      <c r="F1107" s="32" t="s">
+        <v>6</v>
+      </c>
+      <c r="G1107" s="34">
+        <v>3</v>
+      </c>
+      <c r="H1107" s="34" t="s">
+        <v>1898</v>
+      </c>
+      <c r="I1107" s="26" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="1108" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1108" s="35" t="s">
+        <v>64</v>
+      </c>
+      <c r="B1108" s="36">
+        <v>46093</v>
+      </c>
+      <c r="C1108" s="36">
+        <v>46100</v>
+      </c>
+      <c r="D1108" s="48">
+        <v>46160</v>
+      </c>
+      <c r="E1108" s="32" t="s">
+        <v>1899</v>
+      </c>
+      <c r="F1108" s="32" t="s">
+        <v>6</v>
+      </c>
+      <c r="G1108" s="34">
+        <v>3</v>
+      </c>
+      <c r="H1108" s="34" t="s">
+        <v>1900</v>
+      </c>
+      <c r="I1108" s="26" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="1109" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1109" s="35" t="s">
+        <v>267</v>
+      </c>
+      <c r="B1109" s="36">
+        <v>46093</v>
+      </c>
+      <c r="C1109" s="36">
+        <v>46100</v>
+      </c>
+      <c r="D1109" s="48">
+        <v>46160</v>
+      </c>
+      <c r="E1109" s="32" t="s">
+        <v>1901</v>
+      </c>
+      <c r="F1109" s="32" t="s">
+        <v>6</v>
+      </c>
+      <c r="G1109" s="34">
+        <v>3</v>
+      </c>
+      <c r="H1109" s="34" t="s">
+        <v>1902</v>
+      </c>
+      <c r="I1109" s="26" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="1110" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1110" s="35" t="s">
+        <v>267</v>
+      </c>
+      <c r="B1110" s="36">
+        <v>46093</v>
+      </c>
+      <c r="C1110" s="36">
+        <v>46100</v>
+      </c>
+      <c r="D1110" s="48">
+        <v>46160</v>
+      </c>
+      <c r="E1110" s="32" t="s">
+        <v>1903</v>
+      </c>
+      <c r="F1110" s="32" t="s">
+        <v>6</v>
+      </c>
+      <c r="G1110" s="34">
+        <v>2</v>
+      </c>
+      <c r="H1110" s="34" t="s">
+        <v>1904</v>
+      </c>
+      <c r="I1110" s="26" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="1111" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1111" s="35" t="s">
+        <v>267</v>
+      </c>
+      <c r="B1111" s="36">
+        <v>46093</v>
+      </c>
+      <c r="C1111" s="36">
+        <v>46100</v>
+      </c>
+      <c r="D1111" s="48">
+        <v>46160</v>
+      </c>
+      <c r="E1111" s="32" t="s">
+        <v>1905</v>
+      </c>
+      <c r="F1111" s="32" t="s">
+        <v>6</v>
+      </c>
+      <c r="G1111" s="34">
+        <v>3</v>
+      </c>
+      <c r="H1111" s="34" t="s">
+        <v>1906</v>
+      </c>
+      <c r="I1111" s="26" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="1112" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1112" s="35" t="s">
+        <v>267</v>
+      </c>
+      <c r="B1112" s="36">
+        <v>46093</v>
+      </c>
+      <c r="C1112" s="36">
+        <v>46100</v>
+      </c>
+      <c r="D1112" s="48">
+        <v>46160</v>
+      </c>
+      <c r="E1112" s="32" t="s">
+        <v>1907</v>
+      </c>
+      <c r="F1112" s="32" t="s">
+        <v>6</v>
+      </c>
+      <c r="G1112" s="34">
+        <v>3</v>
+      </c>
+      <c r="H1112" s="34" t="s">
+        <v>1908</v>
+      </c>
+      <c r="I1112" s="26" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="1113" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1113" s="35" t="s">
+        <v>267</v>
+      </c>
+      <c r="B1113" s="36">
+        <v>46093</v>
+      </c>
+      <c r="C1113" s="36">
+        <v>46100</v>
+      </c>
+      <c r="D1113" s="48">
+        <v>46160</v>
+      </c>
+      <c r="E1113" s="32" t="s">
+        <v>1909</v>
+      </c>
+      <c r="F1113" s="32" t="s">
+        <v>6</v>
+      </c>
+      <c r="G1113" s="34">
+        <v>4</v>
+      </c>
+      <c r="H1113" s="34" t="s">
+        <v>1910</v>
+      </c>
+      <c r="I1113" s="26" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="1114" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1114" s="35" t="s">
+        <v>267</v>
+      </c>
+      <c r="B1114" s="36">
+        <v>46093</v>
+      </c>
+      <c r="C1114" s="36">
+        <v>46100</v>
+      </c>
+      <c r="D1114" s="48">
+        <v>46160</v>
+      </c>
+      <c r="E1114" s="32" t="s">
+        <v>1911</v>
+      </c>
+      <c r="F1114" s="32" t="s">
+        <v>6</v>
+      </c>
+      <c r="G1114" s="34">
+        <v>3</v>
+      </c>
+      <c r="H1114" s="34" t="s">
+        <v>1912</v>
+      </c>
+      <c r="I1114" s="26" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="1115" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1115" s="35" t="s">
+        <v>267</v>
+      </c>
+      <c r="B1115" s="36">
+        <v>46093</v>
+      </c>
+      <c r="C1115" s="36">
+        <v>46100</v>
+      </c>
+      <c r="D1115" s="48">
+        <v>46160</v>
+      </c>
+      <c r="E1115" s="32" t="s">
+        <v>1913</v>
+      </c>
+      <c r="F1115" s="32" t="s">
+        <v>6</v>
+      </c>
+      <c r="G1115" s="34">
+        <v>3</v>
+      </c>
+      <c r="H1115" s="34" t="s">
+        <v>1914</v>
+      </c>
+      <c r="I1115" s="26" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="1116" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1116" s="35" t="s">
+        <v>267</v>
+      </c>
+      <c r="B1116" s="36">
+        <v>46093</v>
+      </c>
+      <c r="C1116" s="36">
+        <v>46100</v>
+      </c>
+      <c r="D1116" s="48">
+        <v>46160</v>
+      </c>
+      <c r="E1116" s="32" t="s">
+        <v>1915</v>
+      </c>
+      <c r="F1116" s="32" t="s">
+        <v>6</v>
+      </c>
+      <c r="G1116" s="34">
+        <v>3</v>
+      </c>
+      <c r="H1116" s="34" t="s">
+        <v>1916</v>
+      </c>
+      <c r="I1116" s="26" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="1117" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1117" s="35" t="s">
+        <v>267</v>
+      </c>
+      <c r="B1117" s="36">
+        <v>46093</v>
+      </c>
+      <c r="C1117" s="36">
+        <v>46100</v>
+      </c>
+      <c r="D1117" s="48">
+        <v>46160</v>
+      </c>
+      <c r="E1117" s="32" t="s">
+        <v>1917</v>
+      </c>
+      <c r="F1117" s="32" t="s">
+        <v>6</v>
+      </c>
+      <c r="G1117" s="34">
+        <v>4</v>
+      </c>
+      <c r="H1117" s="34" t="s">
+        <v>1918</v>
+      </c>
+      <c r="I1117" s="26" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="1118" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1118" s="35" t="s">
+        <v>71</v>
+      </c>
+      <c r="B1118" s="36">
+        <v>46093</v>
+      </c>
+      <c r="C1118" s="36">
+        <v>46100</v>
+      </c>
+      <c r="D1118" s="48">
+        <v>46160</v>
+      </c>
+      <c r="E1118" s="32" t="s">
+        <v>1919</v>
+      </c>
+      <c r="F1118" s="32" t="s">
+        <v>6</v>
+      </c>
+      <c r="G1118" s="34">
+        <v>2</v>
+      </c>
+      <c r="H1118" s="34" t="s">
+        <v>1920</v>
+      </c>
+      <c r="I1118" s="26" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="1119" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1119" s="35" t="s">
+        <v>74</v>
+      </c>
+      <c r="B1119" s="36">
+        <v>46093</v>
+      </c>
+      <c r="C1119" s="36">
+        <v>46100</v>
+      </c>
+      <c r="D1119" s="48">
+        <v>46160</v>
+      </c>
+      <c r="E1119" s="32" t="s">
+        <v>1921</v>
+      </c>
+      <c r="F1119" s="32" t="s">
+        <v>6</v>
+      </c>
+      <c r="G1119" s="34">
+        <v>2</v>
+      </c>
+      <c r="H1119" s="34" t="s">
+        <v>1922</v>
+      </c>
+      <c r="I1119" s="26" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="1120" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1120" s="35" t="s">
+        <v>5</v>
+      </c>
+      <c r="B1120" s="36">
+        <v>46099</v>
+      </c>
+      <c r="C1120" s="36">
+        <v>46100</v>
+      </c>
+      <c r="D1120" s="48">
+        <v>46162</v>
+      </c>
+      <c r="E1120" s="32" t="s">
+        <v>1923</v>
+      </c>
+      <c r="F1120" s="32" t="s">
+        <v>6</v>
+      </c>
+      <c r="G1120" s="34">
+        <v>97</v>
+      </c>
+      <c r="H1120" s="34" t="s">
+        <v>1924</v>
+      </c>
+      <c r="I1120" s="26" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1121" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1121" s="35" t="s">
+        <v>5</v>
+      </c>
+      <c r="B1121" s="36">
+        <v>46099</v>
+      </c>
+      <c r="C1121" s="36">
+        <v>46100</v>
+      </c>
+      <c r="D1121" s="48">
+        <v>46162</v>
+      </c>
+      <c r="E1121" s="32" t="s">
+        <v>1925</v>
+      </c>
+      <c r="F1121" s="32" t="s">
+        <v>6</v>
+      </c>
+      <c r="G1121" s="34">
+        <v>9</v>
+      </c>
+      <c r="H1121" s="34" t="s">
+        <v>1924</v>
+      </c>
+      <c r="I1121" s="26" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1122" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1122" s="35" t="s">
+        <v>5</v>
+      </c>
+      <c r="B1122" s="36">
+        <v>46099</v>
+      </c>
+      <c r="C1122" s="36">
+        <v>46100</v>
+      </c>
+      <c r="D1122" s="48">
+        <v>46162</v>
+      </c>
+      <c r="E1122" s="32" t="s">
+        <v>1926</v>
+      </c>
+      <c r="F1122" s="32" t="s">
+        <v>6</v>
+      </c>
+      <c r="G1122" s="34">
+        <v>36</v>
+      </c>
+      <c r="H1122" s="34" t="s">
+        <v>1927</v>
+      </c>
+      <c r="I1122" s="26" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1123" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1123" s="35" t="s">
+        <v>5</v>
+      </c>
+      <c r="B1123" s="36">
+        <v>46099</v>
+      </c>
+      <c r="C1123" s="36">
+        <v>46100</v>
+      </c>
+      <c r="D1123" s="48">
+        <v>46162</v>
+      </c>
+      <c r="E1123" s="32" t="s">
+        <v>1928</v>
+      </c>
+      <c r="F1123" s="32" t="s">
+        <v>6</v>
+      </c>
+      <c r="G1123" s="34">
+        <v>43</v>
+      </c>
+      <c r="H1123" s="34" t="s">
+        <v>1929</v>
+      </c>
+      <c r="I1123" s="26" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1124" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1124" s="35" t="s">
+        <v>5</v>
+      </c>
+      <c r="B1124" s="36">
+        <v>46099</v>
+      </c>
+      <c r="C1124" s="36">
+        <v>46100</v>
+      </c>
+      <c r="D1124" s="48">
+        <v>46162</v>
+      </c>
+      <c r="E1124" s="32" t="s">
+        <v>1930</v>
+      </c>
+      <c r="F1124" s="32" t="s">
+        <v>6</v>
+      </c>
+      <c r="G1124" s="34">
+        <v>51</v>
+      </c>
+      <c r="H1124" s="34" t="s">
+        <v>1931</v>
+      </c>
+      <c r="I1124" s="26" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1125" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1125" s="35" t="s">
+        <v>64</v>
+      </c>
+      <c r="B1125" s="36">
+        <v>46101</v>
+      </c>
+      <c r="C1125" s="36">
+        <v>46101</v>
+      </c>
+      <c r="D1125" s="48">
+        <v>46164</v>
+      </c>
+      <c r="E1125" s="32" t="s">
+        <v>1932</v>
+      </c>
+      <c r="F1125" s="32" t="s">
+        <v>54</v>
+      </c>
+      <c r="G1125" s="34">
+        <v>52</v>
+      </c>
+      <c r="H1125" s="34" t="s">
+        <v>1933</v>
+      </c>
+      <c r="I1125" s="26" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="1126" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1126" s="35" t="s">
+        <v>5</v>
+      </c>
+      <c r="B1126" s="36">
+        <v>46099</v>
+      </c>
+      <c r="C1126" s="36">
+        <v>46101</v>
+      </c>
+      <c r="D1126" s="48">
+        <v>46136</v>
+      </c>
+      <c r="E1126" s="32" t="s">
+        <v>1934</v>
+      </c>
+      <c r="F1126" s="32" t="s">
+        <v>6</v>
+      </c>
+      <c r="G1126" s="34">
+        <v>74</v>
+      </c>
+      <c r="H1126" s="34" t="s">
+        <v>1935</v>
+      </c>
+      <c r="I1126" s="26" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="1127" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1127" s="35" t="s">
+        <v>64</v>
+      </c>
+      <c r="B1127" s="36">
+        <v>46100</v>
+      </c>
+      <c r="C1127" s="36">
+        <v>46101</v>
+      </c>
+      <c r="D1127" s="48">
+        <v>46203</v>
+      </c>
+      <c r="E1127" s="32" t="s">
+        <v>1936</v>
+      </c>
+      <c r="F1127" s="32" t="s">
+        <v>6</v>
+      </c>
+      <c r="G1127" s="34">
+        <v>67</v>
+      </c>
+      <c r="H1127" s="34" t="s">
+        <v>1937</v>
+      </c>
+      <c r="I1127" s="26" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="1128" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1128" s="35" t="s">
+        <v>64</v>
+      </c>
+      <c r="B1128" s="36">
+        <v>46100</v>
+      </c>
+      <c r="C1128" s="36">
+        <v>46101</v>
+      </c>
+      <c r="D1128" s="48">
+        <v>46203</v>
+      </c>
+      <c r="E1128" s="32" t="s">
+        <v>1936</v>
+      </c>
+      <c r="F1128" s="32" t="s">
+        <v>6</v>
+      </c>
+      <c r="G1128" s="34">
+        <v>3</v>
+      </c>
+      <c r="H1128" s="34" t="s">
+        <v>1938</v>
+      </c>
+      <c r="I1128" s="26" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="1129" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1129" s="35" t="s">
+        <v>124</v>
+      </c>
+      <c r="B1129" s="36">
+        <v>46100</v>
+      </c>
+      <c r="C1129" s="36">
+        <v>46101</v>
+      </c>
+      <c r="D1129" s="48">
+        <v>46161</v>
+      </c>
+      <c r="E1129" s="32" t="s">
+        <v>282</v>
+      </c>
+      <c r="F1129" s="32" t="s">
+        <v>54</v>
+      </c>
+      <c r="G1129" s="34">
+        <v>44</v>
+      </c>
+      <c r="H1129" s="34" t="s">
+        <v>369</v>
+      </c>
+      <c r="I1129" s="26" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1130" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1130" s="35" t="s">
+        <v>64</v>
+      </c>
+      <c r="B1130" s="36">
+        <v>46101</v>
+      </c>
+      <c r="C1130" s="36">
+        <v>46101</v>
+      </c>
+      <c r="D1130" s="48">
+        <v>46204</v>
+      </c>
+      <c r="E1130" s="32" t="s">
+        <v>258</v>
+      </c>
+      <c r="F1130" s="32" t="s">
+        <v>6</v>
+      </c>
+      <c r="G1130" s="34">
+        <v>23</v>
+      </c>
+      <c r="H1130" s="34" t="s">
+        <v>266</v>
+      </c>
+      <c r="I1130" s="26" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="1131" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1131" s="35" t="s">
+        <v>5</v>
+      </c>
+      <c r="B1131" s="36">
+        <v>46101</v>
+      </c>
+      <c r="C1131" s="36">
+        <v>46104</v>
+      </c>
+      <c r="D1131" s="48">
+        <v>46171</v>
+      </c>
+      <c r="E1131" s="32" t="s">
+        <v>1939</v>
+      </c>
+      <c r="F1131" s="32" t="s">
+        <v>58</v>
+      </c>
+      <c r="G1131" s="34">
+        <v>9</v>
+      </c>
+      <c r="H1131" s="34" t="s">
+        <v>1940</v>
+      </c>
+      <c r="I1131" s="26" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="1132" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1132" s="35" t="s">
+        <v>5</v>
+      </c>
+      <c r="B1132" s="36">
+        <v>46101</v>
+      </c>
+      <c r="C1132" s="36">
+        <v>46104</v>
+      </c>
+      <c r="D1132" s="48">
+        <v>46171</v>
+      </c>
+      <c r="E1132" s="32" t="s">
+        <v>1941</v>
+      </c>
+      <c r="F1132" s="32" t="s">
+        <v>58</v>
+      </c>
+      <c r="G1132" s="34">
+        <v>3</v>
+      </c>
+      <c r="H1132" s="34" t="s">
+        <v>1633</v>
+      </c>
+      <c r="I1132" s="26" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="1133" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1133" s="35" t="s">
+        <v>90</v>
+      </c>
+      <c r="B1133" s="36">
+        <v>46104</v>
+      </c>
+      <c r="C1133" s="36">
+        <v>46104</v>
+      </c>
+      <c r="D1133" s="48">
+        <v>46168</v>
+      </c>
+      <c r="E1133" s="32" t="s">
+        <v>1282</v>
+      </c>
+      <c r="F1133" s="32" t="s">
+        <v>6</v>
+      </c>
+      <c r="G1133" s="34">
+        <v>55</v>
+      </c>
+      <c r="H1133" s="34" t="s">
+        <v>1942</v>
+      </c>
+      <c r="I1133" s="26" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="1134" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1134" s="39" t="s">
+        <v>124</v>
+      </c>
+      <c r="B1134" s="40">
+        <v>46100</v>
+      </c>
+      <c r="C1134" s="40">
+        <v>46104</v>
+      </c>
+      <c r="D1134" s="55">
+        <v>46159</v>
+      </c>
+      <c r="E1134" s="32" t="s">
+        <v>1943</v>
+      </c>
+      <c r="F1134" s="32" t="s">
+        <v>6</v>
+      </c>
+      <c r="G1134" s="34">
+        <v>163</v>
+      </c>
+      <c r="H1134" s="34" t="s">
+        <v>1944</v>
+      </c>
+      <c r="I1134" s="26" t="s">
+        <v>39</v>
       </c>
     </row>
   </sheetData>
@@ -39015,7 +40700,7 @@
           <x14:formula1>
             <xm:f>'Industry List'!$A$1:$A$22</xm:f>
           </x14:formula1>
-          <xm:sqref>I3:I1085</xm:sqref>
+          <xm:sqref>I3:I1134</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -39136,7 +40821,7 @@
   <sheetData>
     <row r="1" spans="1:8" ht="99.75" x14ac:dyDescent="0.25">
       <c r="A1" s="25" t="s">
-        <v>1839</v>
+        <v>1882</v>
       </c>
       <c r="E1"/>
     </row>

</xml_diff>